<commit_message>
s3 done dont need to change
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -11,6 +11,9 @@
     <sheet name="2026-2027" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2025-2027" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="joke" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ict-attendance" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2025-2029" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="1234-1235" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,6 +504,363 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>2025-07-13 00:02:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2025-07-28 13:06:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2025-08-01 08:39:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-08-01 08:44:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2025-08-01 08:51:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2025-08-01 09:02:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2025-08-01 09:04:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:34:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:36:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:38:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:38:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:45:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:00:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:07:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Kirtan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:14:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:19:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:20:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:23:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:23:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:25:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:30:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:32:05</t>
         </is>
       </c>
     </row>
@@ -580,7 +940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -614,6 +974,74 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>2025-07-12 13:02:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>92200133031</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kirtan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:33:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:46:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>92200133031</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kirtan</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:00:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>92200133031</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kirtan</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2025-08-01 22:07:25</t>
         </is>
       </c>
     </row>
@@ -628,7 +1056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -665,6 +1093,456 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-07-28 09:50:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2025-07-28 12:24:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2025-07-28 12:28:48</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ER Number</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Student Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Upload Date &amp; Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>92200133031</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kirtan</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-08-01 11:39:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:18:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:22:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:23:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>92200133031</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kirtan</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:23:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>92200133031</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kirtan</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:26:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:26:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>92200133031</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Kirtan</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:27:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:30:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>92200133031</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Kirtan</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:30:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>92310133005</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Kirtan</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:42:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1234567</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>qwertyu</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:43:15</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ER Number</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Student Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Upload Date &amp; Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Prashant</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:38:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:46:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:49:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>92200133031</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kirtan</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:51:12</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ER Number</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Student Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Upload Date &amp; Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:49:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-08-01 21:50:58</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
code is working to upload img in bucket
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -14,6 +14,7 @@
     <sheet name="ict-attendance" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2025-2029" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="1234-1235" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2021-2022" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1546,4 +1547,52 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ER Number</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Student Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Upload Date &amp; Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-08-06 09:19:22</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
rekognition function is working
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -15,6 +15,7 @@
     <sheet name="2025-2029" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="1234-1235" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2021-2022" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="1234-1234" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1595,4 +1596,69 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ER Number</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Student Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Upload Date &amp; Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>92310133004</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bhargav</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-08-08 11:37:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>92200133013</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Hit</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-08-08 11:45:35</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>